<commit_message>
Corrective action tracker seeded with 12 real actions
</commit_message>
<xml_diff>
--- a/Corrective_Action_Tracker.xlsx
+++ b/Corrective_Action_Tracker.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corrective Action Tracker" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -39,12 +39,17 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="10"/>
+      <sz val="9"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="001e293b"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
@@ -123,18 +128,18 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -156,6 +161,14 @@
         <patternFill patternType="solid">
           <fgColor rgb="00D1FAE5"/>
           <bgColor rgb="00D1FAE5"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00E2E8F0"/>
+          <bgColor rgb="00E2E8F0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -581,17 +594,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1"/>
@@ -606,11 +620,11 @@
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Superior Huntingdon Composites, LLC</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="10" customHeight="1"/>
+          <t>Superior Huntingdon Composites, LLC — 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="8" customHeight="1"/>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
@@ -619,7 +633,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Source</t>
+          <t>Source Inc</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -634,22 +648,27 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
+          <t>Dept</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
           <t>Due Date</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>Days Open</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>Verified Date</t>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>Verify Date</t>
         </is>
       </c>
     </row>
@@ -666,28 +685,31 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Update JSA to include gauging crush roller. Verify E-stop + gauge.</t>
+          <t>Update JSA to include gauging crush roller procedure</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Oven Supvr</t>
+          <t>Bryan</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>02/20/26</t>
+          <t>F team oven</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
+          <t>10/31/26</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="G7" s="4" t="n">
-        <v>251</v>
-      </c>
       <c r="H7" s="4" t="inlineStr"/>
+      <c r="I7" s="4" t="inlineStr"/>
     </row>
     <row r="8" ht="28" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
@@ -697,33 +719,36 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Inc #5</t>
+          <t>Inc #2</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>8D form — forming team pull-back incident.</t>
+          <t>Verify E-stop is installed at crush roller</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Forming Supvr</t>
+          <t>Bryan</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>03/01/26</t>
+          <t>F team oven</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="n">
-        <v>242</v>
+          <t>11/02/26</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
       </c>
       <c r="H8" s="4" t="inlineStr"/>
+      <c r="I8" s="4" t="inlineStr"/>
     </row>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
@@ -731,17 +756,38 @@
           <t>CA-003</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr"/>
-      <c r="C9" s="5" t="inlineStr"/>
-      <c r="D9" s="4" t="inlineStr"/>
-      <c r="E9" s="4" t="inlineStr"/>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Inc #2</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Confirm automated crush roller gauge on order / installed</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Bryan</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>F team oven</t>
+        </is>
+      </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
+          <t>11/06/26</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr"/>
       <c r="H9" s="4" t="inlineStr"/>
+      <c r="I9" s="4" t="inlineStr"/>
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
@@ -749,17 +795,38 @@
           <t>CA-004</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr"/>
-      <c r="C10" s="5" t="inlineStr"/>
-      <c r="D10" s="4" t="inlineStr"/>
-      <c r="E10" s="4" t="inlineStr"/>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Inc #9</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Review eye PPE adequacy for forming/fiberglass work</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Justin</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>C team forming</t>
+        </is>
+      </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
+          <t>11/04/26</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr"/>
       <c r="H10" s="4" t="inlineStr"/>
+      <c r="I10" s="4" t="inlineStr"/>
     </row>
     <row r="11" ht="28" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
@@ -767,38 +834,335 @@
           <t>CA-005</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr"/>
-      <c r="C11" s="5" t="inlineStr"/>
-      <c r="D11" s="4" t="inlineStr"/>
-      <c r="E11" s="4" t="inlineStr"/>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Inc #1</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Complete 8D form - forming team pull-back incident</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Forming Supvr</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Forming</t>
+        </is>
+      </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
+          <t>11/03/26</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr"/>
       <c r="H11" s="4" t="inlineStr"/>
+      <c r="I11" s="4" t="inlineStr"/>
+    </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>CA-006</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Inc #?</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Review hoist reach / ergonomic setup for oven operators</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Bryan</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>F team oven</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>11/09/26</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr"/>
+      <c r="I12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>CA-007</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Inc #4</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Review parking lot ice treatment protocol for snow events</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Facilities</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Parking Lot</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>11/13/26</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr"/>
+      <c r="I13" s="4" t="inlineStr"/>
+    </row>
+    <row r="14" ht="28" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>CA-008</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Multiple</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>New hire orientation checklist rollout (competency-gated)</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Justin</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>11/06/26</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr"/>
+      <c r="I14" s="4" t="inlineStr"/>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>CA-009</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Dry ice blasting trial for oven belt cleaning (cost analysis in progress)</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Justin</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>F team oven</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>11/20/26</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr"/>
+      <c r="I15" s="4" t="inlineStr"/>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>CA-010</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Saw + vacuum extraction for insulation block cutting</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Bryan</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Furnace</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>11/13/26</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr"/>
+      <c r="I16" s="4" t="inlineStr"/>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>CA-011</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Confirm open container drink policy exists / document</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Jodi</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>11/06/26</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr"/>
+      <c r="I17" s="4" t="inlineStr"/>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>CA-012</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Verify SDS QR code system - confirm floor access works</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Justin</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>11/04/26</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr"/>
+      <c r="I18" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A1:H2"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A1:I2"/>
+    <mergeCell ref="A4:I4"/>
+    <mergeCell ref="A3:I3"/>
   </mergeCells>
-  <conditionalFormatting sqref="A7:H11">
+  <conditionalFormatting sqref="A7:I18">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>$F7="Overdue"</formula>
+      <formula>$G7="Overdue"</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="1">
-      <formula>OR($F7="Open",$F7="In Progress")</formula>
+      <formula>OR($G7="Open",$G7="In Progress")</formula>
     </cfRule>
     <cfRule type="expression" priority="3" dxfId="2">
-      <formula>OR($F7="Closed",$F7="Verified")</formula>
+      <formula>OR($G7="Verified",$G7="Closed")</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="3">
+      <formula>$G7="Cancelled"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F7:F11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Open,In Progress,Overdue,Closed,Verified"</formula1>
+    <dataValidation sqref="G7:G18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Open,In Progress,Overdue,Verified,Closed,Cancelled"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -812,49 +1176,51 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-  </cols>
   <sheetData>
     <row r="1"/>
     <row r="2"/>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>CORRECTIVE ACTION SUMMARY</t>
+          <t>CORRECTIVE ACTION STATUS</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>OPEN</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>Overdue</t>
+          <t>OVERDUE</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>Verified</t>
+          <t>VERIFIED</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C6" s="8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E6" s="8" t="n">
         <v>0</v>
@@ -862,18 +1228,21 @@
       <c r="G6" s="8" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="9" t="inlineStr">
-        <is>
-          <t>Update Status on the Corrective Action Tracker tab. Overdue rows turn red automatically.</t>
+      <c r="I6" s="8" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Update the Status column on the Corrective Action Tracker tab. Rows color automatically.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:D2"/>
-    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A1:F2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>